<commit_message>
T-0911: ROW and COLUMN of a multi-cell reference return a vector
Excel-authored evidence: ROW_COLUM.xlsx (upstream, cached values).

Ported-From: ironcalc@b6d34abc

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PPMYgFJYHT9BGwA7Kjzv1p
</commit_message>
<xml_diff>
--- a/crates/rustsheet-xlsx/tests/calc_tests/LOOKUP_AND_REFERENCE/ROW_COLUM.xlsx
+++ b/crates/rustsheet-xlsx/tests/calc_tests/LOOKUP_AND_REFERENCE/ROW_COLUM.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20372"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10927"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8633B9EC-9091-4D34-A9C3-DC2633991AFA}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2395AB79-5B56-1B48-88C1-6C7B6D7976A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12650" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="14260" yWindow="-20980" windowWidth="19220" windowHeight="20980" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ROW_COLUMN" sheetId="1" r:id="rId1"/>
@@ -13,18 +13,52 @@
     <sheet name="INDIRECT" sheetId="4" r:id="rId3"/>
     <sheet name="OTHER" sheetId="2" r:id="rId4"/>
     <sheet name="ROWS_COLUMNS" sheetId="5" r:id="rId5"/>
+    <sheet name="Ranges" sheetId="6" r:id="rId6"/>
+    <sheet name="Sheet2" sheetId="7" r:id="rId7"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="181029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="73">
   <si>
     <t>ROW</t>
   </si>
@@ -231,6 +265,18 @@
   </si>
   <si>
     <t>&lt;= lowercase is valid</t>
+  </si>
+  <si>
+    <t>a</t>
+  </si>
+  <si>
+    <t>b</t>
+  </si>
+  <si>
+    <t>c</t>
+  </si>
+  <si>
+    <t>d</t>
   </si>
 </sst>
 </file>
@@ -609,17 +655,39 @@
 </a:theme>
 </file>
 
+<file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
+<wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
+  <wetp:taskpane dockstate="right" visibility="0" width="350" row="0">
+    <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </wetp:taskpane>
+</wetp:taskpanes>
+</file>
+
+<file path=xl/webextensions/webextension1.xml><?xml version="1.0" encoding="utf-8"?>
+<we:webextension xmlns:we="http://schemas.microsoft.com/office/webextensions/webextension/2010/11" id="{58F842BC-B809-1647-8B4F-54C77F25A70A}">
+  <we:reference id="wa200009404" version="1.0.0.8" store="en-US" storeType="OMEX"/>
+  <we:alternateReferences>
+    <we:reference id="WA200009404" version="1.0.0.8" store="" storeType="OMEX"/>
+  </we:alternateReferences>
+  <we:properties>
+    <we:property name="claude.fileId" value="&quot;c4005590-2396-4b53-b970-1997320c836c&quot;"/>
+  </we:properties>
+  <we:bindings/>
+  <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+</we:webextension>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:XFD24"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="10" max="10" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="18.36328125" customWidth="1"/>
-    <col min="12" max="12" width="22.7265625" customWidth="1"/>
+    <col min="10" max="10" width="9.5" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="18.33203125" customWidth="1"/>
+    <col min="12" max="12" width="22.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:27 16384:16384" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:27 16384:16384" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -643,7 +711,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:27 16384:16384" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:27 16384:16384" x14ac:dyDescent="0.2">
       <c r="A2">
         <f>ROW()</f>
         <v>2</v>
@@ -668,7 +736,7 @@
         <v>#REF!</v>
       </c>
     </row>
-    <row r="3" spans="1:27 16384:16384" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:27 16384:16384" x14ac:dyDescent="0.2">
       <c r="A3">
         <f>ROW()</f>
         <v>3</v>
@@ -693,7 +761,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:27 16384:16384" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:27 16384:16384" x14ac:dyDescent="0.2">
       <c r="A4">
         <f>ROW()</f>
         <v>4</v>
@@ -722,7 +790,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="1:27 16384:16384" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:27 16384:16384" x14ac:dyDescent="0.2">
       <c r="A5">
         <f>ROW()</f>
         <v>5</v>
@@ -747,7 +815,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:27 16384:16384" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:27 16384:16384" x14ac:dyDescent="0.2">
       <c r="A6">
         <f>ROW()</f>
         <v>6</v>
@@ -772,7 +840,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="1:27 16384:16384" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:27 16384:16384" x14ac:dyDescent="0.2">
       <c r="A7">
         <f>ROW()</f>
         <v>7</v>
@@ -789,7 +857,7 @@
         <v>#REF!</v>
       </c>
     </row>
-    <row r="8" spans="1:27 16384:16384" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:27 16384:16384" x14ac:dyDescent="0.2">
       <c r="A8">
         <f>ROW()</f>
         <v>8</v>
@@ -806,7 +874,7 @@
         <v>#REF!</v>
       </c>
     </row>
-    <row r="9" spans="1:27 16384:16384" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:27 16384:16384" x14ac:dyDescent="0.2">
       <c r="A9">
         <f>ROW()</f>
         <v>9</v>
@@ -823,7 +891,7 @@
         <v>#REF!</v>
       </c>
     </row>
-    <row r="10" spans="1:27 16384:16384" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:27 16384:16384" x14ac:dyDescent="0.2">
       <c r="J10" t="s">
         <v>13</v>
       </c>
@@ -836,7 +904,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="11" spans="1:27 16384:16384" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:27 16384:16384" x14ac:dyDescent="0.2">
       <c r="J11" t="s">
         <v>14</v>
       </c>
@@ -849,7 +917,7 @@
         <v>621</v>
       </c>
     </row>
-    <row r="12" spans="1:27 16384:16384" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:27 16384:16384" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>1</v>
       </c>
@@ -894,7 +962,7 @@
         <v>16384</v>
       </c>
     </row>
-    <row r="14" spans="1:27 16384:16384" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:27 16384:16384" x14ac:dyDescent="0.2">
       <c r="A14">
         <f>COLUMN()</f>
         <v>1</v>
@@ -915,7 +983,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="15" spans="1:27 16384:16384" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:27 16384:16384" x14ac:dyDescent="0.2">
       <c r="J15" s="4" t="str">
         <f>"5:5"</f>
         <v>5:5</v>
@@ -929,7 +997,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:27 16384:16384" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:27 16384:16384" x14ac:dyDescent="0.2">
       <c r="J16" t="s">
         <v>57</v>
       </c>
@@ -942,7 +1010,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="17" spans="10:13" x14ac:dyDescent="0.35">
+    <row r="17" spans="10:13" x14ac:dyDescent="0.2">
       <c r="J17" t="s">
         <v>56</v>
       </c>
@@ -955,7 +1023,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="10:13" x14ac:dyDescent="0.35">
+    <row r="18" spans="10:13" x14ac:dyDescent="0.2">
       <c r="J18" t="s">
         <v>58</v>
       </c>
@@ -968,7 +1036,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="19" spans="10:13" x14ac:dyDescent="0.35">
+    <row r="19" spans="10:13" x14ac:dyDescent="0.2">
       <c r="J19" t="s">
         <v>59</v>
       </c>
@@ -981,7 +1049,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="10:13" x14ac:dyDescent="0.35">
+    <row r="20" spans="10:13" x14ac:dyDescent="0.2">
       <c r="J20" t="s">
         <v>60</v>
       </c>
@@ -994,7 +1062,7 @@
         <v>16384</v>
       </c>
     </row>
-    <row r="21" spans="10:13" x14ac:dyDescent="0.35">
+    <row r="21" spans="10:13" x14ac:dyDescent="0.2">
       <c r="J21" t="s">
         <v>61</v>
       </c>
@@ -1007,7 +1075,7 @@
         <v>#REF!</v>
       </c>
     </row>
-    <row r="22" spans="10:13" x14ac:dyDescent="0.35">
+    <row r="22" spans="10:13" x14ac:dyDescent="0.2">
       <c r="J22" s="3" t="s">
         <v>64</v>
       </c>
@@ -1023,7 +1091,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="23" spans="10:13" x14ac:dyDescent="0.35">
+    <row r="23" spans="10:13" x14ac:dyDescent="0.2">
       <c r="J23" t="s">
         <v>65</v>
       </c>
@@ -1036,7 +1104,7 @@
         <v>513</v>
       </c>
     </row>
-    <row r="24" spans="10:13" x14ac:dyDescent="0.35">
+    <row r="24" spans="10:13" x14ac:dyDescent="0.2">
       <c r="J24" t="s">
         <v>66</v>
       </c>
@@ -1060,9 +1128,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AF17D184-111E-423A-A625-82C1BF34E622}">
   <dimension ref="A1:AB54"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A1">
         <v>5</v>
       </c>
@@ -1098,10 +1166,10 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:21" x14ac:dyDescent="0.2">
       <c r="P2" s="1"/>
     </row>
-    <row r="3" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>7</v>
       </c>
@@ -1119,7 +1187,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>5</v>
       </c>
@@ -1130,7 +1198,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>-3</v>
       </c>
@@ -1149,13 +1217,13 @@
         <v>#VALUE!</v>
       </c>
     </row>
-    <row r="6" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:21" x14ac:dyDescent="0.2">
       <c r="P6" s="1"/>
     </row>
-    <row r="7" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:21" x14ac:dyDescent="0.2">
       <c r="P7" s="1"/>
     </row>
-    <row r="8" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:21" x14ac:dyDescent="0.2">
       <c r="P8" s="1">
         <v>13</v>
       </c>
@@ -1164,7 +1232,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="9" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:21" x14ac:dyDescent="0.2">
       <c r="J9">
         <f>H1:O1</f>
         <v>5.7</v>
@@ -1175,7 +1243,7 @@
       </c>
       <c r="P9" s="1"/>
     </row>
-    <row r="10" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:21" x14ac:dyDescent="0.2">
       <c r="B10">
         <f>D1:D1</f>
         <v>0</v>
@@ -1189,14 +1257,14 @@
       </c>
       <c r="P10" s="1"/>
     </row>
-    <row r="11" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:21" x14ac:dyDescent="0.2">
       <c r="M11">
         <f ca="1">SUM(OFFSET(A1,0,7,1,8))</f>
         <v>25.2</v>
       </c>
       <c r="P11" s="1"/>
     </row>
-    <row r="12" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:21" x14ac:dyDescent="0.2">
       <c r="H12" t="s">
         <v>38</v>
       </c>
@@ -1210,21 +1278,21 @@
       </c>
       <c r="P12" s="1"/>
     </row>
-    <row r="13" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:21" x14ac:dyDescent="0.2">
       <c r="P13" s="1"/>
     </row>
-    <row r="14" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:21" x14ac:dyDescent="0.2">
       <c r="P14" s="1"/>
     </row>
-    <row r="15" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:21" x14ac:dyDescent="0.2">
       <c r="P15" s="1"/>
     </row>
-    <row r="16" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:21" x14ac:dyDescent="0.2">
       <c r="P16" s="1">
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.2">
       <c r="J19" t="e">
         <f>P2:P16</f>
         <v>#VALUE!</v>
@@ -1233,12 +1301,12 @@
         <v>39</v>
       </c>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B22" t="s">
         <v>15</v>
       </c>
@@ -1246,7 +1314,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B23" t="s">
         <v>17</v>
       </c>
@@ -1257,7 +1325,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B24" t="s">
         <v>18</v>
       </c>
@@ -1276,7 +1344,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B25" t="s">
         <v>19</v>
       </c>
@@ -1295,7 +1363,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B26" t="s">
         <v>20</v>
       </c>
@@ -1314,7 +1382,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B27" t="s">
         <v>21</v>
       </c>
@@ -1322,7 +1390,7 @@
         <v>-67</v>
       </c>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B28" t="s">
         <v>17</v>
       </c>
@@ -1330,7 +1398,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B29" t="s">
         <v>18</v>
       </c>
@@ -1338,7 +1406,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B30" t="s">
         <v>19</v>
       </c>
@@ -1346,7 +1414,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B31" t="s">
         <v>20</v>
       </c>
@@ -1357,7 +1425,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B32" t="s">
         <v>21</v>
       </c>
@@ -1365,7 +1433,7 @@
         <v>-87</v>
       </c>
     </row>
-    <row r="33" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:28" x14ac:dyDescent="0.2">
       <c r="B33" t="s">
         <v>17</v>
       </c>
@@ -1376,7 +1444,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="34" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:28" x14ac:dyDescent="0.2">
       <c r="B34" t="s">
         <v>18</v>
       </c>
@@ -1384,7 +1452,7 @@
         <v>45.8</v>
       </c>
     </row>
-    <row r="35" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:28" x14ac:dyDescent="0.2">
       <c r="B35" t="s">
         <v>19</v>
       </c>
@@ -1392,7 +1460,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="36" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:28" x14ac:dyDescent="0.2">
       <c r="B36" t="s">
         <v>20</v>
       </c>
@@ -1407,7 +1475,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="37" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:28" x14ac:dyDescent="0.2">
       <c r="B37" t="s">
         <v>21</v>
       </c>
@@ -1425,7 +1493,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="38" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:28" x14ac:dyDescent="0.2">
       <c r="K38" t="e">
         <f ca="1">OFFSET(RS33,2,2, -10, 1)</f>
         <v>#VALUE!</v>
@@ -1437,7 +1505,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="39" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:28" x14ac:dyDescent="0.2">
       <c r="K39" t="e">
         <f ca="1">OFFSET(RS33,2,2, 2, -2)</f>
         <v>#VALUE!</v>
@@ -1452,7 +1520,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="40" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>34</v>
       </c>
@@ -1467,7 +1535,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="41" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>30</v>
       </c>
@@ -1497,7 +1565,7 @@
         <v>-13.5</v>
       </c>
     </row>
-    <row r="42" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>4</v>
       </c>
@@ -1527,7 +1595,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="43" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>4</v>
       </c>
@@ -1563,7 +1631,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="44" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>4</v>
       </c>
@@ -1587,7 +1655,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="45" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>4</v>
       </c>
@@ -1614,7 +1682,7 @@
         <v>65.5</v>
       </c>
     </row>
-    <row r="46" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
         <v>28</v>
       </c>
@@ -1641,7 +1709,7 @@
         <v>58.5</v>
       </c>
     </row>
-    <row r="47" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
         <v>33</v>
       </c>
@@ -1668,7 +1736,7 @@
         <v>#REF!</v>
       </c>
     </row>
-    <row r="48" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
         <v>33</v>
       </c>
@@ -1698,34 +1766,34 @@
         <v>51</v>
       </c>
     </row>
-    <row r="49" spans="11:12" x14ac:dyDescent="0.35">
+    <row r="49" spans="11:12" x14ac:dyDescent="0.2">
       <c r="K49" s="3" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="50" spans="11:12" x14ac:dyDescent="0.35">
+    <row r="50" spans="11:12" x14ac:dyDescent="0.2">
       <c r="K50">
         <f ca="1">SUM(OFFSET(W39,2,2,3,1))</f>
         <v>50</v>
       </c>
     </row>
-    <row r="51" spans="11:12" x14ac:dyDescent="0.35">
+    <row r="51" spans="11:12" x14ac:dyDescent="0.2">
       <c r="K51">
         <f ca="1">SUM(OFFSET(W39,2,2,3,1.2))</f>
         <v>50</v>
       </c>
     </row>
-    <row r="52" spans="11:12" x14ac:dyDescent="0.35">
+    <row r="52" spans="11:12" x14ac:dyDescent="0.2">
       <c r="K52" s="3" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="53" spans="11:12" x14ac:dyDescent="0.35">
+    <row r="53" spans="11:12" x14ac:dyDescent="0.2">
       <c r="K53" s="3" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="54" spans="11:12" x14ac:dyDescent="0.35">
+    <row r="54" spans="11:12" x14ac:dyDescent="0.2">
       <c r="K54" s="2" t="s">
         <v>49</v>
       </c>
@@ -1741,9 +1809,9 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ABDAC406-F3FF-449E-94E7-FD8A17AB8598}">
   <dimension ref="A1:AA34"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>26</v>
       </c>
@@ -1754,7 +1822,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -1771,12 +1839,12 @@
         <v>Cell</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>27</v>
       </c>
       <c r="B3" s="5">
-        <f t="shared" ref="B3:D8" ca="1" si="0">ROW(INDIRECT(A3))</f>
+        <f t="shared" ref="B3:B8" ca="1" si="0">ROW(INDIRECT(A3))</f>
         <v>34</v>
       </c>
       <c r="C3" s="5">
@@ -1788,7 +1856,7 @@
         <v>Hey Jude</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>28</v>
       </c>
@@ -1805,7 +1873,7 @@
         <v>Content of AA23</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>29</v>
       </c>
@@ -1822,7 +1890,7 @@
         <v>#REF!</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B6" s="5" t="e">
         <f t="shared" ca="1" si="0"/>
         <v>#REF!</v>
@@ -1836,7 +1904,7 @@
         <v>#REF!</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B7" s="5" t="e">
         <f t="shared" ca="1" si="0"/>
         <v>#REF!</v>
@@ -1850,7 +1918,7 @@
         <v>#REF!</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>62</v>
       </c>
@@ -1870,12 +1938,12 @@
         <v>63</v>
       </c>
     </row>
-    <row r="23" spans="27:27" x14ac:dyDescent="0.35">
+    <row r="23" spans="27:27" x14ac:dyDescent="0.2">
       <c r="AA23" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="34" spans="19:19" x14ac:dyDescent="0.35">
+    <row r="34" spans="19:19" x14ac:dyDescent="0.2">
       <c r="S34" t="s">
         <v>40</v>
       </c>
@@ -1888,7 +1956,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ADDA4A00-E086-4350-922D-95A6E2BB67AD}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1897,9 +1965,9 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{57980403-3658-4B46-ACC3-124FD43394D7}">
   <dimension ref="A1:H8"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>42</v>
       </c>
@@ -1907,7 +1975,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2">
         <f>ROWS(A1)</f>
         <v>1</v>
@@ -1920,7 +1988,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3">
         <f>ROWS(AA23)</f>
         <v>1</v>
@@ -1938,7 +2006,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A4">
         <f>ROWS(H2:Q12)</f>
         <v>11</v>
@@ -1956,7 +2024,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A5">
         <f>ROWS(OTHER!B3:AC29)</f>
         <v>27</v>
@@ -1974,7 +2042,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A6" s="5">
         <f>ROWS(C:C)</f>
         <v>1048576</v>
@@ -2000,7 +2068,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7" s="5">
         <f>ROWS(14:14)</f>
         <v>1</v>
@@ -2010,7 +2078,7 @@
         <v>16384</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A8" s="5">
         <f>ROWS($AB:$AAA)</f>
         <v>1048576</v>
@@ -2018,6 +2086,160 @@
       <c r="B8" s="5">
         <f>COLUMNS($AB:$AAA)</f>
         <v>676</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2192BF6D-C4B7-E54D-9608-19D34EB00ED3}">
+  <dimension ref="A1:I18"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A1" cm="1">
+        <f t="array" ref="A1:C1">COLUMN(C2:E4)</f>
+        <v>3</v>
+      </c>
+      <c r="B1">
+        <v>4</v>
+      </c>
+      <c r="C1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="F3" cm="1">
+        <f t="array" ref="F3">SUM(ROW(C2:C4))</f>
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="F4" cm="1">
+        <f t="array" ref="F4">SUM(COLUMN(C2:E2))</f>
+        <v>12</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="F5" cm="1">
+        <f t="array" ref="F5">SUM(ROW(C2:C4)*COLUMN(C2:E2))</f>
+        <v>108</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A9" cm="1">
+        <f t="array" ref="A9:A11">ROW(C2:E4)</f>
+        <v>2</v>
+      </c>
+      <c r="H9" cm="1">
+        <f t="array" aca="1" ref="H9:H11" ca="1">ROW(OFFSET(C2,1,0,3,1))</f>
+        <v>3</v>
+      </c>
+      <c r="I9" cm="1">
+        <f t="array" aca="1" ref="I9" ca="1">SUM(COLUMN(OFFSET(C2,0,1,1,3)))</f>
+        <v>15</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A10">
+        <v>3</v>
+      </c>
+      <c r="E10" cm="1">
+        <f t="array" ref="E10">ROW(C7:E7)</f>
+        <v>7</v>
+      </c>
+      <c r="H10">
+        <f ca="1"/>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A11">
+        <v>4</v>
+      </c>
+      <c r="E11" cm="1">
+        <f t="array" ref="E11">COLUMN(C7:C9)</f>
+        <v>3</v>
+      </c>
+      <c r="H11">
+        <f ca="1"/>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A18" cm="1">
+        <f t="array" ref="A18">MAX(ROW(Sheet2!B:B))</f>
+        <v>1048576</v>
+      </c>
+      <c r="B18" cm="1">
+        <f t="array" ref="B18">MAX(COLUMN(Sheet2!7:7))</f>
+        <v>16384</v>
+      </c>
+      <c r="C18" cm="1">
+        <f t="array" ref="C18">MAX((Sheet2!B:B&lt;&gt;"")*ROW(Sheet2!B:B))</f>
+        <v>7</v>
+      </c>
+      <c r="D18" cm="1">
+        <f t="array" ref="D18">MAX((Sheet2!7:7&lt;&gt;"")*COLUMN(Sheet2!7:7))</f>
+        <v>2</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F3D8D184-9542-E24E-9DA6-BBB402BE130B}">
+  <dimension ref="A1:C7"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A1" cm="1">
+        <f t="array" ref="A1">MAX((C1:C20&lt;&gt;"")*ROW(C1:C20))</f>
+        <v>6</v>
+      </c>
+      <c r="B1" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A2" cm="1">
+        <f t="array" ref="A2">MAX((A3:J3&lt;&gt;"")*COLUMN(A3:J3))</f>
+        <v>3</v>
+      </c>
+      <c r="B2" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="C3" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="B4" t="s">
+        <v>71</v>
+      </c>
+      <c r="C4" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="C5" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="C6" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="B7" t="s">
+        <v>72</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
T-0911: ROW/COLUMN of multi-cell references return vectors (ported ironcalc b6d34abc)
Ported-From: ironcalc@b6d34abc

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PPMYgFJYHT9BGwA7Kjzv1p
</commit_message>
<xml_diff>
--- a/crates/rustsheet-xlsx/tests/calc_tests/LOOKUP_AND_REFERENCE/ROW_COLUM.xlsx
+++ b/crates/rustsheet-xlsx/tests/calc_tests/LOOKUP_AND_REFERENCE/ROW_COLUM.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20372"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10927"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8633B9EC-9091-4D34-A9C3-DC2633991AFA}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2395AB79-5B56-1B48-88C1-6C7B6D7976A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12650" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="14260" yWindow="-20980" windowWidth="19220" windowHeight="20980" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ROW_COLUMN" sheetId="1" r:id="rId1"/>
@@ -13,18 +13,52 @@
     <sheet name="INDIRECT" sheetId="4" r:id="rId3"/>
     <sheet name="OTHER" sheetId="2" r:id="rId4"/>
     <sheet name="ROWS_COLUMNS" sheetId="5" r:id="rId5"/>
+    <sheet name="Ranges" sheetId="6" r:id="rId6"/>
+    <sheet name="Sheet2" sheetId="7" r:id="rId7"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="181029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="73">
   <si>
     <t>ROW</t>
   </si>
@@ -231,6 +265,18 @@
   </si>
   <si>
     <t>&lt;= lowercase is valid</t>
+  </si>
+  <si>
+    <t>a</t>
+  </si>
+  <si>
+    <t>b</t>
+  </si>
+  <si>
+    <t>c</t>
+  </si>
+  <si>
+    <t>d</t>
   </si>
 </sst>
 </file>
@@ -609,17 +655,39 @@
 </a:theme>
 </file>
 
+<file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
+<wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
+  <wetp:taskpane dockstate="right" visibility="0" width="350" row="0">
+    <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </wetp:taskpane>
+</wetp:taskpanes>
+</file>
+
+<file path=xl/webextensions/webextension1.xml><?xml version="1.0" encoding="utf-8"?>
+<we:webextension xmlns:we="http://schemas.microsoft.com/office/webextensions/webextension/2010/11" id="{58F842BC-B809-1647-8B4F-54C77F25A70A}">
+  <we:reference id="wa200009404" version="1.0.0.8" store="en-US" storeType="OMEX"/>
+  <we:alternateReferences>
+    <we:reference id="WA200009404" version="1.0.0.8" store="" storeType="OMEX"/>
+  </we:alternateReferences>
+  <we:properties>
+    <we:property name="claude.fileId" value="&quot;c4005590-2396-4b53-b970-1997320c836c&quot;"/>
+  </we:properties>
+  <we:bindings/>
+  <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+</we:webextension>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:XFD24"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="10" max="10" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="18.36328125" customWidth="1"/>
-    <col min="12" max="12" width="22.7265625" customWidth="1"/>
+    <col min="10" max="10" width="9.5" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="18.33203125" customWidth="1"/>
+    <col min="12" max="12" width="22.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:27 16384:16384" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:27 16384:16384" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -643,7 +711,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:27 16384:16384" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:27 16384:16384" x14ac:dyDescent="0.2">
       <c r="A2">
         <f>ROW()</f>
         <v>2</v>
@@ -668,7 +736,7 @@
         <v>#REF!</v>
       </c>
     </row>
-    <row r="3" spans="1:27 16384:16384" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:27 16384:16384" x14ac:dyDescent="0.2">
       <c r="A3">
         <f>ROW()</f>
         <v>3</v>
@@ -693,7 +761,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:27 16384:16384" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:27 16384:16384" x14ac:dyDescent="0.2">
       <c r="A4">
         <f>ROW()</f>
         <v>4</v>
@@ -722,7 +790,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="1:27 16384:16384" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:27 16384:16384" x14ac:dyDescent="0.2">
       <c r="A5">
         <f>ROW()</f>
         <v>5</v>
@@ -747,7 +815,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:27 16384:16384" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:27 16384:16384" x14ac:dyDescent="0.2">
       <c r="A6">
         <f>ROW()</f>
         <v>6</v>
@@ -772,7 +840,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="1:27 16384:16384" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:27 16384:16384" x14ac:dyDescent="0.2">
       <c r="A7">
         <f>ROW()</f>
         <v>7</v>
@@ -789,7 +857,7 @@
         <v>#REF!</v>
       </c>
     </row>
-    <row r="8" spans="1:27 16384:16384" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:27 16384:16384" x14ac:dyDescent="0.2">
       <c r="A8">
         <f>ROW()</f>
         <v>8</v>
@@ -806,7 +874,7 @@
         <v>#REF!</v>
       </c>
     </row>
-    <row r="9" spans="1:27 16384:16384" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:27 16384:16384" x14ac:dyDescent="0.2">
       <c r="A9">
         <f>ROW()</f>
         <v>9</v>
@@ -823,7 +891,7 @@
         <v>#REF!</v>
       </c>
     </row>
-    <row r="10" spans="1:27 16384:16384" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:27 16384:16384" x14ac:dyDescent="0.2">
       <c r="J10" t="s">
         <v>13</v>
       </c>
@@ -836,7 +904,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="11" spans="1:27 16384:16384" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:27 16384:16384" x14ac:dyDescent="0.2">
       <c r="J11" t="s">
         <v>14</v>
       </c>
@@ -849,7 +917,7 @@
         <v>621</v>
       </c>
     </row>
-    <row r="12" spans="1:27 16384:16384" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:27 16384:16384" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>1</v>
       </c>
@@ -894,7 +962,7 @@
         <v>16384</v>
       </c>
     </row>
-    <row r="14" spans="1:27 16384:16384" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:27 16384:16384" x14ac:dyDescent="0.2">
       <c r="A14">
         <f>COLUMN()</f>
         <v>1</v>
@@ -915,7 +983,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="15" spans="1:27 16384:16384" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:27 16384:16384" x14ac:dyDescent="0.2">
       <c r="J15" s="4" t="str">
         <f>"5:5"</f>
         <v>5:5</v>
@@ -929,7 +997,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:27 16384:16384" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:27 16384:16384" x14ac:dyDescent="0.2">
       <c r="J16" t="s">
         <v>57</v>
       </c>
@@ -942,7 +1010,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="17" spans="10:13" x14ac:dyDescent="0.35">
+    <row r="17" spans="10:13" x14ac:dyDescent="0.2">
       <c r="J17" t="s">
         <v>56</v>
       </c>
@@ -955,7 +1023,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="10:13" x14ac:dyDescent="0.35">
+    <row r="18" spans="10:13" x14ac:dyDescent="0.2">
       <c r="J18" t="s">
         <v>58</v>
       </c>
@@ -968,7 +1036,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="19" spans="10:13" x14ac:dyDescent="0.35">
+    <row r="19" spans="10:13" x14ac:dyDescent="0.2">
       <c r="J19" t="s">
         <v>59</v>
       </c>
@@ -981,7 +1049,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="10:13" x14ac:dyDescent="0.35">
+    <row r="20" spans="10:13" x14ac:dyDescent="0.2">
       <c r="J20" t="s">
         <v>60</v>
       </c>
@@ -994,7 +1062,7 @@
         <v>16384</v>
       </c>
     </row>
-    <row r="21" spans="10:13" x14ac:dyDescent="0.35">
+    <row r="21" spans="10:13" x14ac:dyDescent="0.2">
       <c r="J21" t="s">
         <v>61</v>
       </c>
@@ -1007,7 +1075,7 @@
         <v>#REF!</v>
       </c>
     </row>
-    <row r="22" spans="10:13" x14ac:dyDescent="0.35">
+    <row r="22" spans="10:13" x14ac:dyDescent="0.2">
       <c r="J22" s="3" t="s">
         <v>64</v>
       </c>
@@ -1023,7 +1091,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="23" spans="10:13" x14ac:dyDescent="0.35">
+    <row r="23" spans="10:13" x14ac:dyDescent="0.2">
       <c r="J23" t="s">
         <v>65</v>
       </c>
@@ -1036,7 +1104,7 @@
         <v>513</v>
       </c>
     </row>
-    <row r="24" spans="10:13" x14ac:dyDescent="0.35">
+    <row r="24" spans="10:13" x14ac:dyDescent="0.2">
       <c r="J24" t="s">
         <v>66</v>
       </c>
@@ -1060,9 +1128,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AF17D184-111E-423A-A625-82C1BF34E622}">
   <dimension ref="A1:AB54"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A1">
         <v>5</v>
       </c>
@@ -1098,10 +1166,10 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:21" x14ac:dyDescent="0.2">
       <c r="P2" s="1"/>
     </row>
-    <row r="3" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>7</v>
       </c>
@@ -1119,7 +1187,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>5</v>
       </c>
@@ -1130,7 +1198,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>-3</v>
       </c>
@@ -1149,13 +1217,13 @@
         <v>#VALUE!</v>
       </c>
     </row>
-    <row r="6" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:21" x14ac:dyDescent="0.2">
       <c r="P6" s="1"/>
     </row>
-    <row r="7" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:21" x14ac:dyDescent="0.2">
       <c r="P7" s="1"/>
     </row>
-    <row r="8" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:21" x14ac:dyDescent="0.2">
       <c r="P8" s="1">
         <v>13</v>
       </c>
@@ -1164,7 +1232,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="9" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:21" x14ac:dyDescent="0.2">
       <c r="J9">
         <f>H1:O1</f>
         <v>5.7</v>
@@ -1175,7 +1243,7 @@
       </c>
       <c r="P9" s="1"/>
     </row>
-    <row r="10" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:21" x14ac:dyDescent="0.2">
       <c r="B10">
         <f>D1:D1</f>
         <v>0</v>
@@ -1189,14 +1257,14 @@
       </c>
       <c r="P10" s="1"/>
     </row>
-    <row r="11" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:21" x14ac:dyDescent="0.2">
       <c r="M11">
         <f ca="1">SUM(OFFSET(A1,0,7,1,8))</f>
         <v>25.2</v>
       </c>
       <c r="P11" s="1"/>
     </row>
-    <row r="12" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:21" x14ac:dyDescent="0.2">
       <c r="H12" t="s">
         <v>38</v>
       </c>
@@ -1210,21 +1278,21 @@
       </c>
       <c r="P12" s="1"/>
     </row>
-    <row r="13" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:21" x14ac:dyDescent="0.2">
       <c r="P13" s="1"/>
     </row>
-    <row r="14" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:21" x14ac:dyDescent="0.2">
       <c r="P14" s="1"/>
     </row>
-    <row r="15" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:21" x14ac:dyDescent="0.2">
       <c r="P15" s="1"/>
     </row>
-    <row r="16" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:21" x14ac:dyDescent="0.2">
       <c r="P16" s="1">
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.2">
       <c r="J19" t="e">
         <f>P2:P16</f>
         <v>#VALUE!</v>
@@ -1233,12 +1301,12 @@
         <v>39</v>
       </c>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B22" t="s">
         <v>15</v>
       </c>
@@ -1246,7 +1314,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B23" t="s">
         <v>17</v>
       </c>
@@ -1257,7 +1325,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B24" t="s">
         <v>18</v>
       </c>
@@ -1276,7 +1344,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B25" t="s">
         <v>19</v>
       </c>
@@ -1295,7 +1363,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B26" t="s">
         <v>20</v>
       </c>
@@ -1314,7 +1382,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B27" t="s">
         <v>21</v>
       </c>
@@ -1322,7 +1390,7 @@
         <v>-67</v>
       </c>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B28" t="s">
         <v>17</v>
       </c>
@@ -1330,7 +1398,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B29" t="s">
         <v>18</v>
       </c>
@@ -1338,7 +1406,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B30" t="s">
         <v>19</v>
       </c>
@@ -1346,7 +1414,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B31" t="s">
         <v>20</v>
       </c>
@@ -1357,7 +1425,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B32" t="s">
         <v>21</v>
       </c>
@@ -1365,7 +1433,7 @@
         <v>-87</v>
       </c>
     </row>
-    <row r="33" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:28" x14ac:dyDescent="0.2">
       <c r="B33" t="s">
         <v>17</v>
       </c>
@@ -1376,7 +1444,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="34" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:28" x14ac:dyDescent="0.2">
       <c r="B34" t="s">
         <v>18</v>
       </c>
@@ -1384,7 +1452,7 @@
         <v>45.8</v>
       </c>
     </row>
-    <row r="35" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:28" x14ac:dyDescent="0.2">
       <c r="B35" t="s">
         <v>19</v>
       </c>
@@ -1392,7 +1460,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="36" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:28" x14ac:dyDescent="0.2">
       <c r="B36" t="s">
         <v>20</v>
       </c>
@@ -1407,7 +1475,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="37" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:28" x14ac:dyDescent="0.2">
       <c r="B37" t="s">
         <v>21</v>
       </c>
@@ -1425,7 +1493,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="38" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:28" x14ac:dyDescent="0.2">
       <c r="K38" t="e">
         <f ca="1">OFFSET(RS33,2,2, -10, 1)</f>
         <v>#VALUE!</v>
@@ -1437,7 +1505,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="39" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:28" x14ac:dyDescent="0.2">
       <c r="K39" t="e">
         <f ca="1">OFFSET(RS33,2,2, 2, -2)</f>
         <v>#VALUE!</v>
@@ -1452,7 +1520,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="40" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>34</v>
       </c>
@@ -1467,7 +1535,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="41" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>30</v>
       </c>
@@ -1497,7 +1565,7 @@
         <v>-13.5</v>
       </c>
     </row>
-    <row r="42" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>4</v>
       </c>
@@ -1527,7 +1595,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="43" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>4</v>
       </c>
@@ -1563,7 +1631,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="44" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>4</v>
       </c>
@@ -1587,7 +1655,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="45" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>4</v>
       </c>
@@ -1614,7 +1682,7 @@
         <v>65.5</v>
       </c>
     </row>
-    <row r="46" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
         <v>28</v>
       </c>
@@ -1641,7 +1709,7 @@
         <v>58.5</v>
       </c>
     </row>
-    <row r="47" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
         <v>33</v>
       </c>
@@ -1668,7 +1736,7 @@
         <v>#REF!</v>
       </c>
     </row>
-    <row r="48" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
         <v>33</v>
       </c>
@@ -1698,34 +1766,34 @@
         <v>51</v>
       </c>
     </row>
-    <row r="49" spans="11:12" x14ac:dyDescent="0.35">
+    <row r="49" spans="11:12" x14ac:dyDescent="0.2">
       <c r="K49" s="3" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="50" spans="11:12" x14ac:dyDescent="0.35">
+    <row r="50" spans="11:12" x14ac:dyDescent="0.2">
       <c r="K50">
         <f ca="1">SUM(OFFSET(W39,2,2,3,1))</f>
         <v>50</v>
       </c>
     </row>
-    <row r="51" spans="11:12" x14ac:dyDescent="0.35">
+    <row r="51" spans="11:12" x14ac:dyDescent="0.2">
       <c r="K51">
         <f ca="1">SUM(OFFSET(W39,2,2,3,1.2))</f>
         <v>50</v>
       </c>
     </row>
-    <row r="52" spans="11:12" x14ac:dyDescent="0.35">
+    <row r="52" spans="11:12" x14ac:dyDescent="0.2">
       <c r="K52" s="3" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="53" spans="11:12" x14ac:dyDescent="0.35">
+    <row r="53" spans="11:12" x14ac:dyDescent="0.2">
       <c r="K53" s="3" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="54" spans="11:12" x14ac:dyDescent="0.35">
+    <row r="54" spans="11:12" x14ac:dyDescent="0.2">
       <c r="K54" s="2" t="s">
         <v>49</v>
       </c>
@@ -1741,9 +1809,9 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ABDAC406-F3FF-449E-94E7-FD8A17AB8598}">
   <dimension ref="A1:AA34"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>26</v>
       </c>
@@ -1754,7 +1822,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -1771,12 +1839,12 @@
         <v>Cell</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>27</v>
       </c>
       <c r="B3" s="5">
-        <f t="shared" ref="B3:D8" ca="1" si="0">ROW(INDIRECT(A3))</f>
+        <f t="shared" ref="B3:B8" ca="1" si="0">ROW(INDIRECT(A3))</f>
         <v>34</v>
       </c>
       <c r="C3" s="5">
@@ -1788,7 +1856,7 @@
         <v>Hey Jude</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>28</v>
       </c>
@@ -1805,7 +1873,7 @@
         <v>Content of AA23</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>29</v>
       </c>
@@ -1822,7 +1890,7 @@
         <v>#REF!</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B6" s="5" t="e">
         <f t="shared" ca="1" si="0"/>
         <v>#REF!</v>
@@ -1836,7 +1904,7 @@
         <v>#REF!</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B7" s="5" t="e">
         <f t="shared" ca="1" si="0"/>
         <v>#REF!</v>
@@ -1850,7 +1918,7 @@
         <v>#REF!</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>62</v>
       </c>
@@ -1870,12 +1938,12 @@
         <v>63</v>
       </c>
     </row>
-    <row r="23" spans="27:27" x14ac:dyDescent="0.35">
+    <row r="23" spans="27:27" x14ac:dyDescent="0.2">
       <c r="AA23" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="34" spans="19:19" x14ac:dyDescent="0.35">
+    <row r="34" spans="19:19" x14ac:dyDescent="0.2">
       <c r="S34" t="s">
         <v>40</v>
       </c>
@@ -1888,7 +1956,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ADDA4A00-E086-4350-922D-95A6E2BB67AD}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1897,9 +1965,9 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{57980403-3658-4B46-ACC3-124FD43394D7}">
   <dimension ref="A1:H8"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>42</v>
       </c>
@@ -1907,7 +1975,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2">
         <f>ROWS(A1)</f>
         <v>1</v>
@@ -1920,7 +1988,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3">
         <f>ROWS(AA23)</f>
         <v>1</v>
@@ -1938,7 +2006,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A4">
         <f>ROWS(H2:Q12)</f>
         <v>11</v>
@@ -1956,7 +2024,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A5">
         <f>ROWS(OTHER!B3:AC29)</f>
         <v>27</v>
@@ -1974,7 +2042,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A6" s="5">
         <f>ROWS(C:C)</f>
         <v>1048576</v>
@@ -2000,7 +2068,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7" s="5">
         <f>ROWS(14:14)</f>
         <v>1</v>
@@ -2010,7 +2078,7 @@
         <v>16384</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A8" s="5">
         <f>ROWS($AB:$AAA)</f>
         <v>1048576</v>
@@ -2018,6 +2086,160 @@
       <c r="B8" s="5">
         <f>COLUMNS($AB:$AAA)</f>
         <v>676</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2192BF6D-C4B7-E54D-9608-19D34EB00ED3}">
+  <dimension ref="A1:I18"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A1" cm="1">
+        <f t="array" ref="A1:C1">COLUMN(C2:E4)</f>
+        <v>3</v>
+      </c>
+      <c r="B1">
+        <v>4</v>
+      </c>
+      <c r="C1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="F3" cm="1">
+        <f t="array" ref="F3">SUM(ROW(C2:C4))</f>
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="F4" cm="1">
+        <f t="array" ref="F4">SUM(COLUMN(C2:E2))</f>
+        <v>12</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="F5" cm="1">
+        <f t="array" ref="F5">SUM(ROW(C2:C4)*COLUMN(C2:E2))</f>
+        <v>108</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A9" cm="1">
+        <f t="array" ref="A9:A11">ROW(C2:E4)</f>
+        <v>2</v>
+      </c>
+      <c r="H9" cm="1">
+        <f t="array" aca="1" ref="H9:H11" ca="1">ROW(OFFSET(C2,1,0,3,1))</f>
+        <v>3</v>
+      </c>
+      <c r="I9" cm="1">
+        <f t="array" aca="1" ref="I9" ca="1">SUM(COLUMN(OFFSET(C2,0,1,1,3)))</f>
+        <v>15</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A10">
+        <v>3</v>
+      </c>
+      <c r="E10" cm="1">
+        <f t="array" ref="E10">ROW(C7:E7)</f>
+        <v>7</v>
+      </c>
+      <c r="H10">
+        <f ca="1"/>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A11">
+        <v>4</v>
+      </c>
+      <c r="E11" cm="1">
+        <f t="array" ref="E11">COLUMN(C7:C9)</f>
+        <v>3</v>
+      </c>
+      <c r="H11">
+        <f ca="1"/>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A18" cm="1">
+        <f t="array" ref="A18">MAX(ROW(Sheet2!B:B))</f>
+        <v>1048576</v>
+      </c>
+      <c r="B18" cm="1">
+        <f t="array" ref="B18">MAX(COLUMN(Sheet2!7:7))</f>
+        <v>16384</v>
+      </c>
+      <c r="C18" cm="1">
+        <f t="array" ref="C18">MAX((Sheet2!B:B&lt;&gt;"")*ROW(Sheet2!B:B))</f>
+        <v>7</v>
+      </c>
+      <c r="D18" cm="1">
+        <f t="array" ref="D18">MAX((Sheet2!7:7&lt;&gt;"")*COLUMN(Sheet2!7:7))</f>
+        <v>2</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F3D8D184-9542-E24E-9DA6-BBB402BE130B}">
+  <dimension ref="A1:C7"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A1" cm="1">
+        <f t="array" ref="A1">MAX((C1:C20&lt;&gt;"")*ROW(C1:C20))</f>
+        <v>6</v>
+      </c>
+      <c r="B1" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A2" cm="1">
+        <f t="array" ref="A2">MAX((A3:J3&lt;&gt;"")*COLUMN(A3:J3))</f>
+        <v>3</v>
+      </c>
+      <c r="B2" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="C3" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="B4" t="s">
+        <v>71</v>
+      </c>
+      <c r="C4" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="C5" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="C6" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="B7" t="s">
+        <v>72</v>
       </c>
     </row>
   </sheetData>

</xml_diff>